<commit_message>
feat: student can enter average score
</commit_message>
<xml_diff>
--- a/data/study_data.xlsx
+++ b/data/study_data.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="69">
   <si>
     <t>id</t>
   </si>
@@ -211,6 +211,18 @@
   </si>
   <si>
     <t>myScore</t>
+  </si>
+  <si>
+    <t>averageScore</t>
+  </si>
+  <si>
+    <t>1780737666251</t>
+  </si>
+  <si>
+    <t>2026-06-09T00:00:00.000Z</t>
+  </si>
+  <si>
+    <t>test</t>
   </si>
 </sst>
 </file>
@@ -246,10 +258,6 @@
     </font>
     <font>
       <b/>
-      <color theme="1"/>
-      <family val="2"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -301,9 +309,7 @@
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1218,16 +1224,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="5" width="12.43357142857143" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" ht="17.25" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -1243,8 +1243,32 @@
       <c r="E1" s="10" t="s">
         <v>64</v>
       </c>
+      <c r="F1" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2">
+        <v>20</v>
+      </c>
+      <c r="F2">
+        <v>19</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: user should type user name when sign up
</commit_message>
<xml_diff>
--- a/data/study_data.xlsx
+++ b/data/study_data.xlsx
@@ -10,30 +10,78 @@
     <sheet sheetId="1" name="StudySessions" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Environment" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Exams" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Users" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Groups" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="69">
-  <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>subject</t>
-  </si>
-  <si>
-    <t>startTime</t>
-  </si>
-  <si>
-    <t>endTime</t>
-  </si>
-  <si>
-    <t>durationMinutes</t>
-  </si>
-  <si>
-    <t>focusScore</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="109">
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>id</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>subject</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>startTime</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>endTime</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>durationMinutes</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>focusScore</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>studentId</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
   </si>
   <si>
     <t>1780222800338</t>
@@ -42,10 +90,23 @@
     <t>物理</t>
   </si>
   <si>
-    <t>2026-05-31T10:17:01.781Z</t>
-  </si>
-  <si>
-    <t>2026-05-31T10:20:00.114Z</t>
+    <r>
+      <t>2026-06-01T10:17:01.781Z</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>2026-06-01T10:20:00.114Z</t>
+    </r>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> B10303123</t>
   </si>
   <si>
     <t>1780223026016</t>
@@ -54,10 +115,20 @@
     <t>數學</t>
   </si>
   <si>
-    <t>2026-05-31T10:22:12.096Z</t>
-  </si>
-  <si>
-    <t>2026-05-31T10:23:45.962Z</t>
+    <r>
+      <t>2026-06-01T10:22:12.096Z</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>2026-06-01T10:23:45.962Z</t>
+    </r>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>4</t>
   </si>
   <si>
     <t>1780224753627</t>
@@ -66,28 +137,49 @@
     <t>化學</t>
   </si>
   <si>
-    <t>2026-05-31T10:51:25.934Z</t>
-  </si>
-  <si>
-    <t>2026-05-31T10:52:33.583Z</t>
+    <r>
+      <t>2026-06-01T10:51:25.934Z</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>2026-06-01T10:52:33.583Z</t>
+    </r>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>7</t>
   </si>
   <si>
     <t>1780225608547</t>
   </si>
   <si>
-    <t>2026-05-31T11:04:36.090Z</t>
-  </si>
-  <si>
-    <t>2026-05-31T11:06:48.292Z</t>
+    <r>
+      <t>2026-06-01T11:04:36.090Z</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>2026-06-01T11:06:48.292Z</t>
+    </r>
   </si>
   <si>
     <t>1780226187527</t>
   </si>
   <si>
-    <t>2026-05-31T11:15:06.243Z</t>
-  </si>
-  <si>
-    <t>2026-05-31T11:16:27.310Z</t>
+    <r>
+      <t>2026-06-01T11:15:06.243Z</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>2026-06-01T11:16:27.310Z</t>
+    </r>
+  </si>
+  <si>
+    <t>8</t>
   </si>
   <si>
     <t>1780226479639</t>
@@ -96,10 +188,65 @@
     <t>英文</t>
   </si>
   <si>
-    <t>2026-05-31T11:16:43.060Z</t>
-  </si>
-  <si>
-    <t>2026-05-31T11:21:19.458Z</t>
+    <r>
+      <t>2026-06-01T11:16:43.060Z</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>2026-06-01T11:21:19.458Z</t>
+    </r>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>1780743802235</t>
+  </si>
+  <si>
+    <r>
+      <t>2026-06-01T11:00:58.802Z</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>2026-06-01T11:03:22.200Z</t>
+    </r>
+  </si>
+  <si>
+    <t>B10303123</t>
+  </si>
+  <si>
+    <t>1780744037113</t>
+  </si>
+  <si>
+    <t>國文</t>
+  </si>
+  <si>
+    <t>2026-06-06T11:03:36.252Z</t>
+  </si>
+  <si>
+    <r>
+      <t>2026-06-06T11:07:17.085Z</t>
+    </r>
+  </si>
+  <si>
+    <t>1780744552856</t>
+  </si>
+  <si>
+    <t>2026-06-06T11:14:43.653Z</t>
+  </si>
+  <si>
+    <t>2026-06-06T11:15:52.837Z</t>
+  </si>
+  <si>
+    <t>1780744870983</t>
+  </si>
+  <si>
+    <t>2026-06-06T11:19:58.142Z</t>
+  </si>
+  <si>
+    <t>2026-06-06T11:21:10.960Z</t>
   </si>
   <si>
     <t>date</t>
@@ -204,16 +351,36 @@
     <t>2026-06-30</t>
   </si>
   <si>
-    <t>examDate</t>
-  </si>
-  <si>
-    <t>examName</t>
-  </si>
-  <si>
-    <t>myScore</t>
-  </si>
-  <si>
-    <t>averageScore</t>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>examDate</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>examName</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>myScore</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>averageScore</t>
+    </r>
   </si>
   <si>
     <t>1780737666251</t>
@@ -223,13 +390,68 @@
   </si>
   <si>
     <t>test</t>
+  </si>
+  <si>
+    <t>1780745016135</t>
+  </si>
+  <si>
+    <t>2026-06-11T00:00:00.000Z</t>
+  </si>
+  <si>
+    <t>期中考</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>password</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>displayName</t>
+    </r>
+  </si>
+  <si>
+    <t>1234</t>
+  </si>
+  <si>
+    <t>Serena</t>
+  </si>
+  <si>
+    <t>chich1234</t>
+  </si>
+  <si>
+    <t>chich</t>
+  </si>
+  <si>
+    <t>groupId</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>createdBy</t>
+  </si>
+  <si>
+    <t>members</t>
+  </si>
+  <si>
+    <t>MO5QJ3</t>
+  </si>
+  <si>
+    <t>Test</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -240,12 +462,6 @@
     <font>
       <b/>
       <color rgb="FF000000"/>
-      <family val="2"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <color theme="1"/>
       <family val="2"/>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -280,36 +496,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -615,154 +828,269 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="12.43357142857143" customWidth="1"/>
-    <col min="3" max="3" width="30.290714285714284" customWidth="1"/>
-    <col min="4" max="4" width="35.14785714285715" customWidth="1"/>
-    <col min="5" max="5" width="26.14785714285714" style="1" customWidth="1"/>
-    <col min="6" max="6" width="12.43357142857143" style="1" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="19.5" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" ht="19.5" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" ht="17.25" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" ht="17.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" ht="17.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="G8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9" t="s">
+        <v>46</v>
+      </c>
+      <c r="E9">
+        <v>4</v>
+      </c>
+      <c r="F9">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="G9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="4">
+      <c r="C10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D10" t="s">
+        <v>49</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
         <v>3</v>
       </c>
-      <c r="F2" s="4">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" ht="17.25" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" s="4">
+      <c r="G10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11">
         <v>1</v>
       </c>
-      <c r="F3" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="1">
-        <v>0</v>
-      </c>
-      <c r="F4" s="1">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="1">
-        <v>0</v>
-      </c>
-      <c r="F5" s="1">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E6" s="1">
-        <v>1</v>
-      </c>
-      <c r="F6" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="1">
-        <v>2</v>
-      </c>
-      <c r="F7" s="1">
-        <v>3</v>
+      <c r="F11">
+        <v>9</v>
+      </c>
+      <c r="G11" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -779,441 +1107,441 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.43357142857143" customWidth="1"/>
-    <col min="2" max="2" width="12.43357142857143" style="5" customWidth="1"/>
-    <col min="3" max="4" width="12.43357142857143" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.43357142857143" style="1" customWidth="1"/>
+    <col min="3" max="4" width="12.43357142857143" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>31</v>
+      <c r="A1" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="2" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" s="7">
+        <v>57</v>
+      </c>
+      <c r="B2" s="6">
         <v>33.4</v>
       </c>
-      <c r="C2" s="8">
+      <c r="C2" s="7">
         <v>85</v>
       </c>
-      <c r="D2" s="8">
+      <c r="D2" s="7">
         <v>774</v>
       </c>
     </row>
     <row r="3" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B3" s="7">
+        <v>58</v>
+      </c>
+      <c r="B3" s="6">
         <v>26.5</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="7">
         <v>86</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="7">
         <v>432</v>
       </c>
     </row>
     <row r="4" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" s="7">
+        <v>59</v>
+      </c>
+      <c r="B4" s="6">
         <v>30.5</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="7">
         <v>85</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="7">
         <v>469</v>
       </c>
     </row>
     <row r="5" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5" s="8">
+        <v>60</v>
+      </c>
+      <c r="B5" s="7">
         <v>29</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="7">
         <v>63</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="7">
         <v>382</v>
       </c>
     </row>
     <row r="6" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B6" s="7">
+        <v>61</v>
+      </c>
+      <c r="B6" s="6">
         <v>29.6</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="7">
         <v>68</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="7">
         <v>510</v>
       </c>
     </row>
     <row r="7" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B7" s="8">
+        <v>62</v>
+      </c>
+      <c r="B7" s="7">
         <v>31</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="7">
         <v>85</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="7">
         <v>648</v>
       </c>
     </row>
     <row r="8" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" s="7">
+        <v>63</v>
+      </c>
+      <c r="B8" s="6">
         <v>27.3</v>
       </c>
-      <c r="C8" s="8">
+      <c r="C8" s="7">
         <v>65</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="7">
         <v>467</v>
       </c>
     </row>
     <row r="9" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B9" s="7">
+        <v>64</v>
+      </c>
+      <c r="B9" s="6">
         <v>28.6</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="7">
         <v>75</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="7">
         <v>730</v>
       </c>
     </row>
     <row r="10" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>40</v>
-      </c>
-      <c r="B10" s="7">
+        <v>65</v>
+      </c>
+      <c r="B10" s="6">
         <v>30.3</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="7">
         <v>77</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="7">
         <v>579</v>
       </c>
     </row>
     <row r="11" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B11" s="7">
+        <v>66</v>
+      </c>
+      <c r="B11" s="6">
         <v>33.8</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="7">
         <v>74</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="7">
         <v>434</v>
       </c>
     </row>
     <row r="12" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>42</v>
-      </c>
-      <c r="B12" s="7">
+        <v>67</v>
+      </c>
+      <c r="B12" s="6">
         <v>32.6</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="7">
         <v>76</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="7">
         <v>682</v>
       </c>
     </row>
     <row r="13" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>43</v>
-      </c>
-      <c r="B13" s="7">
+        <v>68</v>
+      </c>
+      <c r="B13" s="6">
         <v>27.4</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="7">
         <v>69</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="7">
         <v>418</v>
       </c>
     </row>
     <row r="14" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>44</v>
-      </c>
-      <c r="B14" s="8">
+        <v>69</v>
+      </c>
+      <c r="B14" s="7">
         <v>34</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="7">
         <v>65</v>
       </c>
-      <c r="D14" s="8">
+      <c r="D14" s="7">
         <v>682</v>
       </c>
     </row>
     <row r="15" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>45</v>
-      </c>
-      <c r="B15" s="7">
+        <v>70</v>
+      </c>
+      <c r="B15" s="6">
         <v>32.5</v>
       </c>
-      <c r="C15" s="8">
+      <c r="C15" s="7">
         <v>83</v>
       </c>
-      <c r="D15" s="8">
+      <c r="D15" s="7">
         <v>534</v>
       </c>
     </row>
     <row r="16" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>46</v>
-      </c>
-      <c r="B16" s="7">
+        <v>71</v>
+      </c>
+      <c r="B16" s="6">
         <v>29.5</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="7">
         <v>74</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="7">
         <v>351</v>
       </c>
     </row>
     <row r="17" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>47</v>
-      </c>
-      <c r="B17" s="7">
+        <v>72</v>
+      </c>
+      <c r="B17" s="6">
         <v>33.4</v>
       </c>
-      <c r="C17" s="8">
+      <c r="C17" s="7">
         <v>61</v>
       </c>
-      <c r="D17" s="8">
+      <c r="D17" s="7">
         <v>572</v>
       </c>
     </row>
     <row r="18" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>48</v>
-      </c>
-      <c r="B18" s="7">
+        <v>73</v>
+      </c>
+      <c r="B18" s="6">
         <v>29.5</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="7">
         <v>74</v>
       </c>
-      <c r="D18" s="8">
+      <c r="D18" s="7">
         <v>339</v>
       </c>
     </row>
     <row r="19" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B19" s="7">
+        <v>74</v>
+      </c>
+      <c r="B19" s="6">
         <v>31.2</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="7">
         <v>62</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="7">
         <v>467</v>
       </c>
     </row>
     <row r="20" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>50</v>
-      </c>
-      <c r="B20" s="7">
+        <v>75</v>
+      </c>
+      <c r="B20" s="6">
         <v>28.6</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20" s="7">
         <v>64</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="7">
         <v>229</v>
       </c>
     </row>
     <row r="21" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>51</v>
-      </c>
-      <c r="B21" s="7">
+        <v>76</v>
+      </c>
+      <c r="B21" s="6">
         <v>32.1</v>
       </c>
-      <c r="C21" s="8">
+      <c r="C21" s="7">
         <v>65</v>
       </c>
-      <c r="D21" s="8">
+      <c r="D21" s="7">
         <v>724</v>
       </c>
     </row>
     <row r="22" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>52</v>
-      </c>
-      <c r="B22" s="7">
+        <v>77</v>
+      </c>
+      <c r="B22" s="6">
         <v>30.4</v>
       </c>
-      <c r="C22" s="8">
+      <c r="C22" s="7">
         <v>71</v>
       </c>
-      <c r="D22" s="8">
+      <c r="D22" s="7">
         <v>745</v>
       </c>
     </row>
     <row r="23" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>53</v>
-      </c>
-      <c r="B23" s="7">
+        <v>78</v>
+      </c>
+      <c r="B23" s="6">
         <v>31.3</v>
       </c>
-      <c r="C23" s="8">
+      <c r="C23" s="7">
         <v>87</v>
       </c>
-      <c r="D23" s="8">
+      <c r="D23" s="7">
         <v>704</v>
       </c>
     </row>
     <row r="24" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>54</v>
-      </c>
-      <c r="B24" s="7">
+        <v>79</v>
+      </c>
+      <c r="B24" s="6">
         <v>29.4</v>
       </c>
-      <c r="C24" s="8">
+      <c r="C24" s="7">
         <v>80</v>
       </c>
-      <c r="D24" s="8">
+      <c r="D24" s="7">
         <v>875</v>
       </c>
     </row>
     <row r="25" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>55</v>
-      </c>
-      <c r="B25" s="7">
+        <v>80</v>
+      </c>
+      <c r="B25" s="6">
         <v>27.1</v>
       </c>
-      <c r="C25" s="8">
+      <c r="C25" s="7">
         <v>56</v>
       </c>
-      <c r="D25" s="8">
+      <c r="D25" s="7">
         <v>559</v>
       </c>
     </row>
     <row r="26" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>56</v>
-      </c>
-      <c r="B26" s="7">
+        <v>81</v>
+      </c>
+      <c r="B26" s="6">
         <v>28.6</v>
       </c>
-      <c r="C26" s="8">
+      <c r="C26" s="7">
         <v>57</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="7">
         <v>382</v>
       </c>
     </row>
     <row r="27" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>57</v>
-      </c>
-      <c r="B27" s="8">
+        <v>82</v>
+      </c>
+      <c r="B27" s="7">
         <v>30</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C27" s="7">
         <v>67</v>
       </c>
-      <c r="D27" s="8">
+      <c r="D27" s="7">
         <v>647</v>
       </c>
     </row>
     <row r="28" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>58</v>
-      </c>
-      <c r="B28" s="8">
+        <v>83</v>
+      </c>
+      <c r="B28" s="7">
         <v>26</v>
       </c>
-      <c r="C28" s="8">
+      <c r="C28" s="7">
         <v>83</v>
       </c>
-      <c r="D28" s="8">
+      <c r="D28" s="7">
         <v>341</v>
       </c>
     </row>
     <row r="29" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>59</v>
-      </c>
-      <c r="B29" s="7">
+        <v>84</v>
+      </c>
+      <c r="B29" s="6">
         <v>27.3</v>
       </c>
-      <c r="C29" s="8">
+      <c r="C29" s="7">
         <v>82</v>
       </c>
-      <c r="D29" s="8">
+      <c r="D29" s="7">
         <v>811</v>
       </c>
     </row>
     <row r="30" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>60</v>
-      </c>
-      <c r="B30" s="7">
+        <v>85</v>
+      </c>
+      <c r="B30" s="6">
         <v>29.4</v>
       </c>
-      <c r="C30" s="8">
+      <c r="C30" s="7">
         <v>87</v>
       </c>
-      <c r="D30" s="8">
+      <c r="D30" s="7">
         <v>737</v>
       </c>
     </row>
     <row r="31" ht="17.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>61</v>
-      </c>
-      <c r="B31" s="7">
+        <v>86</v>
+      </c>
+      <c r="B31" s="6">
         <v>33.9</v>
       </c>
-      <c r="C31" s="8">
+      <c r="C31" s="7">
         <v>72</v>
       </c>
-      <c r="D31" s="9">
+      <c r="D31" s="8">
         <v>526</v>
       </c>
     </row>
@@ -1224,47 +1552,189 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="D1" s="10" t="s">
+      <c r="B1" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E1" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>91</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>92</v>
       </c>
       <c r="C2" t="s">
-        <v>68</v>
+        <v>93</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="E2">
         <v>20</v>
       </c>
       <c r="F2">
         <v>19</v>
+      </c>
+      <c r="G2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3">
+        <v>99</v>
+      </c>
+      <c r="F3">
+        <v>80</v>
+      </c>
+      <c r="G3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>